<commit_message>
Add L28 (Le Bourget) via data/extra_listings.csv
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/Paris_konaklama_v2.xlsx
+++ b/out/Paris_konaklama_v2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Açıklama" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İlanlar'!$A$1:$AA$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İlanlar'!$A$1:$AA$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA26"/>
+  <dimension ref="A1:AA27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -749,28 +749,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>L25</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Booking</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Güzel daire, balkon ve otopark</t>
+          <t>Entire apartment F3 next to RER B Antony</t>
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>45616</v>
+        <v>59000</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>39629</v>
+        <v>58606</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>2</v>
@@ -785,59 +785,57 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 tek kişilik yatak Oturma odası 1 kanepe</t>
+          <t>Yatak Odası 1: 1 çift kişilik yatak; Yatak Odası 2: 2 tek kişilik yatak</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>4.95</v>
+        <v>8</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Argenteuil</t>
+          <t>Les Baconnets</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>TRAIN J</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T3" s="2" t="n">
-        <v>1170</v>
+        <v>390</v>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>yaklaşık</t>
+          <t>kesin</t>
         </is>
       </c>
       <c r="V3" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Argenteuil, Fransa</t>
+          <t>4 Rue Maurice Brouard, 92160 Antony, Fransa</t>
         </is>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+          <t>10 Kasım 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="3" t="inlineStr">
         <is>
-          <t>Ulaşım ve durak bilgisi teyit edilmeli.</t>
+          <t>25 yaş altı check-in yapılamıyor; 200 € nakit depozito; rezervasyon talebi; 10 Kasım öncesi ücretsiz iptal koşulunu kontrol et.</t>
         </is>
       </c>
       <c r="Z3" s="5" t="inlineStr">
@@ -856,7 +854,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -963,11 +961,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>L18</t>
+          <t>L25</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -977,14 +975,14 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>70047</v>
+          <t>Güzel daire, balkon ve otopark</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>45616</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>60723</v>
+        <v>39629</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>2</v>
@@ -995,43 +993,43 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 tek kişilik yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>4.88</v>
+        <v>4.95</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>11.4</v>
+        <v>12.5</v>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Le Bourget</t>
+          <t>Argenteuil</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>RER B, TRAM 11</t>
+          <t>TRAIN J</t>
         </is>
       </c>
       <c r="T5" s="2" t="n">
-        <v>260</v>
+        <v>1170</v>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
@@ -1040,7 +1038,7 @@
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
+          <t>Tüm kiralık konut, Argenteuil, Fransa</t>
         </is>
       </c>
       <c r="W5" s="3" t="inlineStr">
@@ -1048,14 +1046,10 @@
           <t>Ücretsiz iptal son gün: 12 Kasım</t>
         </is>
       </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>14:00-22:00</t>
-        </is>
-      </c>
+      <c r="X5" s="2" t="n"/>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t>Önceki tabloda A02; misafir yorumuna göre RER 3 dk; 12 Kasım ücretsiz iptal.</t>
+          <t>Ulaşım ve durak bilgisi teyit edilmeli.</t>
         </is>
       </c>
       <c r="Z5" s="5" t="inlineStr">
@@ -1074,11 +1068,11 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>L24</t>
+          <t>L17</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1088,17 +1082,17 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Paris 13'te 3 yatak odalı daire 800 m - WIFI</t>
+          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>74542</v>
+        <v>71934</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>64861</v>
+        <v>61880</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -1106,43 +1100,43 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 2 tek kişilik yatak 2. yatak odası 2 tek kişilik yatak 3. yatak odası 1 çift kişilik yatak Oturma odası 1 kanepe</t>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 çift kişilik yatak</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>4.7</v>
+        <v>4.63</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>Le Kremlin - Bicêtre</t>
+          <t>Laplace</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>METRO 7</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T6" s="2" t="n">
-        <v>270</v>
+        <v>130</v>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
@@ -1151,18 +1145,22 @@
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t>Tüm otel olanakları sunan möbleli daire, Le Kremlin-Bicêtre, Fransa</t>
+          <t>Tüm villa, Arcueil, Fransa</t>
         </is>
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="n"/>
+          <t>Ücretsiz iptal son gün: 30 Ekim</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>15:00-23:00</t>
+        </is>
+      </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>Bütçeye çok yakın; ödeme aşamasında toplamı teyit et.</t>
+          <t>Önceki tabloda A07; Laplace RER 2–3 dk; Ağustos 2026’da evin durumu hakkında olumsuz değerlendirme var.</t>
         </is>
       </c>
       <c r="Z6" s="5" t="inlineStr">
@@ -1181,28 +1179,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L18</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Booking</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Entire apartment F3 next to RER B Antony</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>59000</v>
+          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>70047</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>58606</v>
+        <v>60723</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>2</v>
@@ -1213,61 +1211,67 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 1 çift kişilik yatak; Yatak Odası 2: 2 tek kişilik yatak</t>
+          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>8</v>
+        <v>4.88</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N7" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P7" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n">
-        <v>37</v>
-      </c>
       <c r="Q7" s="2" t="n">
-        <v>12.3</v>
+        <v>11.4</v>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>Les Baconnets</t>
+          <t>Le Bourget</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>RER B, TRAM 11</t>
         </is>
       </c>
       <c r="T7" s="2" t="n">
-        <v>390</v>
+        <v>260</v>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>kesin</t>
+          <t>yaklaşık</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t>4 Rue Maurice Brouard, 92160 Antony, Fransa</t>
+          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
         </is>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>10 Kasım 2026 öncesinde ücretsiz iptal</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="n"/>
+          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>14:00-22:00</t>
+        </is>
+      </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>25 yaş altı check-in yapılamıyor; 200 € nakit depozito; rezervasyon talebi; 10 Kasım öncesi ücretsiz iptal koşulunu kontrol et.</t>
+          <t>Önceki tabloda A02; misafir yorumuna göre RER 3 dk; 12 Kasım ücretsiz iptal.</t>
         </is>
       </c>
       <c r="Z7" s="5" t="inlineStr">
@@ -1286,11 +1290,11 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>L17</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1300,61 +1304,57 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
+          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>71934</v>
+        <v>66832</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>61880</v>
+        <v>58136</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>onaylı</t>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>doğrulanmalı</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 çift kişilik yatak</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K8" s="3" t="n"/>
       <c r="L8" s="2" t="n">
-        <v>4.63</v>
+        <v>4.9</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>Laplace</t>
+          <t>La Croix de Berny</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>RER B, TRAM 10</t>
         </is>
       </c>
       <c r="T8" s="2" t="n">
-        <v>130</v>
+        <v>290</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
@@ -1363,22 +1363,14 @@
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>Tüm villa, Arcueil, Fransa</t>
-        </is>
-      </c>
-      <c r="W8" s="3" t="inlineStr">
-        <is>
-          <t>Ücretsiz iptal son gün: 30 Ekim</t>
-        </is>
-      </c>
-      <c r="X8" s="2" t="inlineStr">
-        <is>
-          <t>15:00-23:00</t>
-        </is>
-      </c>
+          <t>Tüm site içi konut, Antony, Fransa</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="2" t="n"/>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>Önceki tabloda A07; Laplace RER 2–3 dk; Ağustos 2026’da evin durumu hakkında olumsuz değerlendirme var.</t>
+          <t>Arama fiyatı 9 gece için tüm ücretler dâhil gösteriliyor; oda ve koşullar incelenmeli.</t>
         </is>
       </c>
       <c r="Z8" s="5" t="inlineStr">
@@ -1397,7 +1389,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -1508,11 +1500,11 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>L14</t>
+          <t>L13</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1522,14 +1514,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Aile için T3, ulaşım, mağazalar</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>72595</v>
+          <t>Appartement T3 Antony/Orly 10 dk.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>62401</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>62914</v>
+        <v>54348</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>2</v>
@@ -1544,26 +1536,26 @@
       </c>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>4.79</v>
+        <v>4.57</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="O10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>5.3</v>
+        <v>8.5</v>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>Arcueil - Cachan</t>
+          <t>Parc de Sceaux</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1572,7 +1564,7 @@
         </is>
       </c>
       <c r="T10" s="2" t="n">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
@@ -1581,18 +1573,22 @@
       </c>
       <c r="V10" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Cachan, Fransa</t>
+          <t>Tüm kiralık konut, Antony, Fransa</t>
         </is>
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 8 Kasım</t>
-        </is>
-      </c>
-      <c r="X10" s="2" t="n"/>
+          <t>24 saat süreyle ücretsiz iptal.</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>17:00-23:00</t>
+        </is>
+      </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t>Önceki tabloda A06; RER B 5 dk yürüme; giriş en erken 20.00.</t>
+          <t>RER B Parc de Sceaux: ilanda 5 dakika deniyor, yürüyüş olup olmadığı teyit edilmeli.</t>
         </is>
       </c>
       <c r="Z10" s="5" t="inlineStr">
@@ -1611,11 +1607,11 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>L12</t>
+          <t>L16</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1625,57 +1621,61 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
+          <t>Montmartre'ın göbeğinde ferah ve aydınlık daire</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>66832</v>
+        <v>66801</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>58136</v>
+        <v>57852</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>doğrulanmalı</t>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>onaylı</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K11" s="3" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="n">
-        <v>4.9</v>
+        <v>4.44</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>129</v>
+        <v>9</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>10</v>
+        <v>4.3</v>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>La Croix de Berny</t>
+          <t>Abbesses</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>RER B, TRAM 10</t>
+          <t>METRO 12</t>
         </is>
       </c>
       <c r="T11" s="2" t="n">
-        <v>290</v>
+        <v>210</v>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
@@ -1684,14 +1684,22 @@
       </c>
       <c r="V11" s="3" t="inlineStr">
         <is>
-          <t>Tüm site içi konut, Antony, Fransa</t>
-        </is>
-      </c>
-      <c r="W11" s="3" t="n"/>
-      <c r="X11" s="2" t="n"/>
+          <t>Tüm kiralık konut, Paris, Fransa</t>
+        </is>
+      </c>
+      <c r="W11" s="3" t="inlineStr">
+        <is>
+          <t>24 saat süreyle ücretsiz iptal.</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>15:00-21:00</t>
+        </is>
+      </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>Arama fiyatı 9 gece için tüm ücretler dâhil gösteriliyor; oda ve koşullar incelenmeli.</t>
+          <t>Oda düzeni, yorumlar ve ulaşım doğrulanmalı.</t>
         </is>
       </c>
       <c r="Z11" s="5" t="inlineStr">
@@ -1710,11 +1718,11 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>L16</t>
+          <t>L28</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1724,14 +1732,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Montmartre'ın göbeğinde ferah ve aydınlık daire</t>
+          <t>L'Écrin Parisien • T3 Design • Le Bourget • CDG Havalimanı</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>66801</v>
+        <v>72174</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>57852</v>
+        <v>62442</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>2</v>
@@ -1742,43 +1750,41 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
+          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>4.44</v>
+        <v>4.94</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P12" s="2" t="n">
-        <v>36</v>
-      </c>
+      <c r="P12" s="2" t="n"/>
       <c r="Q12" s="2" t="n">
-        <v>4.3</v>
+        <v>11.6</v>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>Abbesses</t>
+          <t>Le Bourget</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>METRO 12</t>
+          <t>RER B, TRAM 11</t>
         </is>
       </c>
       <c r="T12" s="2" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
@@ -1787,22 +1793,18 @@
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Paris, Fransa</t>
+          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
         </is>
       </c>
       <c r="W12" s="3" t="inlineStr">
         <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X12" s="2" t="inlineStr">
-        <is>
-          <t>15:00-21:00</t>
-        </is>
-      </c>
+          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="n"/>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>Oda düzeni, yorumlar ve ulaşım doğrulanmalı.</t>
+          <t>Kullanıcı sonradan ekledi (28.10.2026).</t>
         </is>
       </c>
       <c r="Z12" s="5" t="inlineStr">
@@ -1821,11 +1823,11 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>L13</t>
+          <t>L15</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1835,48 +1837,52 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Appartement T3 Antony/Orly 10 dk.</t>
+          <t>Daire F3 - Arcueil</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>62401</v>
+        <v>62927</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>54348</v>
+        <v>54442</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>doğrulanmalı</t>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>onaylı</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" s="3" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>1. yatak odası 1 tek kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="n">
-        <v>4.57</v>
+        <v>4.44</v>
       </c>
       <c r="M13" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>8.5</v>
+        <v>4.9</v>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>Parc de Sceaux</t>
+          <t>Arcueil - Cachan</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -1885,7 +1891,7 @@
         </is>
       </c>
       <c r="T13" s="2" t="n">
-        <v>360</v>
+        <v>520</v>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
@@ -1894,22 +1900,18 @@
       </c>
       <c r="V13" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Antony, Fransa</t>
+          <t>Tüm kiralık konut, Arcueil, Fransa</t>
         </is>
       </c>
       <c r="W13" s="3" t="inlineStr">
         <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X13" s="2" t="inlineStr">
-        <is>
-          <t>17:00-23:00</t>
-        </is>
-      </c>
+          <t>Ücretsiz iptal son gün: 8 Kasım</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="n"/>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>RER B Parc de Sceaux: ilanda 5 dakika deniyor, yürüyüş olup olmadığı teyit edilmeli.</t>
+          <t>İki ayrı oda; yorumlarda gece izinsiz giriş veya giriş denemesi iddiaları var; koşulları ve istasyonu teyit et.</t>
         </is>
       </c>
       <c r="Z13" s="5" t="inlineStr">
@@ -1928,11 +1930,11 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>L15</t>
+          <t>L24</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1942,17 +1944,17 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Daire F3 - Arcueil</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>62927</v>
+          <t>Paris 13'te 3 yatak odalı daire 800 m - WIFI</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>74542</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>54442</v>
+        <v>64861</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1960,43 +1962,43 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 tek kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
+          <t>1. yatak odası 2 tek kişilik yatak 2. yatak odası 2 tek kişilik yatak 3. yatak odası 1 çift kişilik yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>4.44</v>
+        <v>4.7</v>
       </c>
       <c r="M14" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>4.9</v>
+        <v>4</v>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>Arcueil - Cachan</t>
+          <t>Le Kremlin - Bicêtre</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>METRO 7</t>
         </is>
       </c>
       <c r="T14" s="2" t="n">
-        <v>520</v>
+        <v>270</v>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
@@ -2005,18 +2007,18 @@
       </c>
       <c r="V14" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Arcueil, Fransa</t>
+          <t>Tüm otel olanakları sunan möbleli daire, Le Kremlin-Bicêtre, Fransa</t>
         </is>
       </c>
       <c r="W14" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 8 Kasım</t>
+          <t>24 saat süreyle ücretsiz iptal.</t>
         </is>
       </c>
       <c r="X14" s="2" t="n"/>
       <c r="Y14" s="3" t="inlineStr">
         <is>
-          <t>İki ayrı oda; yorumlarda gece izinsiz giriş veya giriş denemesi iddiaları var; koşulları ve istasyonu teyit et.</t>
+          <t>Bütçeye çok yakın; ödeme aşamasında toplamı teyit et.</t>
         </is>
       </c>
       <c r="Z14" s="5" t="inlineStr">
@@ -2035,11 +2037,11 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>L22</t>
+          <t>L14</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2049,61 +2051,57 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Geniş daire, 2 yatak odası/7 kişi - Nogent-sur-Marne</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>63659</v>
+          <t>Aile için T3, ulaşım, mağazalar</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>72595</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>59755</v>
+        <v>62914</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>şüpheli</t>
+          <t>doğrulanmalı</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak, 1 tek kişilik yatak Oturma odası 1 kanepe</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K15" s="3" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>5</v>
+        <v>4.79</v>
       </c>
       <c r="M15" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>10.9</v>
+        <v>5.3</v>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>Nogent - Le Perreux</t>
+          <t>Arcueil - Cachan</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>RER E</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T15" s="2" t="n">
-        <v>440</v>
+        <v>370</v>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
@@ -2112,22 +2110,18 @@
       </c>
       <c r="V15" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Nogent-sur-Marne, Fransa</t>
+          <t>Tüm kiralık konut, Cachan, Fransa</t>
         </is>
       </c>
       <c r="W15" s="3" t="inlineStr">
         <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X15" s="2" t="inlineStr">
-        <is>
-          <t>16:00-23:00</t>
-        </is>
-      </c>
+          <t>Ücretsiz iptal son gün: 8 Kasım</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="n"/>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t>Odalardan biri asma katta görünüyor; kapalı oda olup olmadığı teyit edilmeli.</t>
+          <t>Önceki tabloda A06; RER B 5 dk yürüme; giriş en erken 20.00.</t>
         </is>
       </c>
       <c r="Z15" s="5" t="inlineStr">
@@ -2146,11 +2140,11 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>L26</t>
+          <t>L22</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2160,14 +2154,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Appartement neuf</t>
+          <t>Geniş daire, 2 yatak odası/7 kişi - Nogent-sur-Marne</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>57612</v>
+        <v>63659</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>50298</v>
+        <v>59755</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>2</v>
@@ -2178,43 +2172,43 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Yaşam alanı 1 kraliçe yatak, 1 çift kişilik yatak, 1 kanepe, 1 beşik</t>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak, 1 tek kişilik yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L16" s="2" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>8.300000000000001</v>
+        <v>10.9</v>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>Maisons-Alfort - Alfortville</t>
+          <t>Nogent - Le Perreux</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>RER D</t>
+          <t>RER E</t>
         </is>
       </c>
       <c r="T16" s="2" t="n">
-        <v>810</v>
+        <v>440</v>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
@@ -2223,7 +2217,7 @@
       </c>
       <c r="V16" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Alfortville, Fransa</t>
+          <t>Tüm kiralık konut, Nogent-sur-Marne, Fransa</t>
         </is>
       </c>
       <c r="W16" s="3" t="inlineStr">
@@ -2231,10 +2225,14 @@
           <t>24 saat süreyle ücretsiz iptal.</t>
         </is>
       </c>
-      <c r="X16" s="2" t="n"/>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>16:00-23:00</t>
+        </is>
+      </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
-          <t>Oda, konum ve koşullar doğrulanmalı.</t>
+          <t>Odalardan biri asma katta görünüyor; kapalı oda olup olmadığı teyit edilmeli.</t>
         </is>
       </c>
       <c r="Z16" s="5" t="inlineStr">
@@ -2253,93 +2251,95 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L26</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Booking</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>T2 Coteau CACHAN</t>
+          <t>Appartement neuf</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>46000</v>
+        <v>57612</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>46590</v>
+        <v>50298</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>yok</t>
+          <t>şüpheli</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 1 çift kişilik yatak ve 1 büyük çift kişilik yatak</t>
+          <t>Yaşam alanı 1 kraliçe yatak, 1 çift kişilik yatak, 1 kanepe, 1 beşik</t>
         </is>
       </c>
       <c r="L17" s="2" t="n">
-        <v>9</v>
+        <v>4.8</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N17" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="O17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>5.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>Villejuif - Gustave Roussy</t>
+          <t>Maisons-Alfort - Alfortville</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>METRO 14</t>
+          <t>RER D</t>
         </is>
       </c>
       <c r="T17" s="2" t="n">
-        <v>820</v>
+        <v>810</v>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>kesin</t>
+          <t>yaklaşık</t>
         </is>
       </c>
       <c r="V17" s="3" t="inlineStr">
         <is>
-          <t>Appartement A 6 Boulevard de la Vanne, 94230 Cachan, Fransa</t>
+          <t>Tüm kiralık konut, Alfortville, Fransa</t>
         </is>
       </c>
       <c r="W17" s="3" t="inlineStr">
         <is>
-          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
+          <t>24 saat süreyle ücretsiz iptal.</t>
         </is>
       </c>
       <c r="X17" s="2" t="n"/>
       <c r="Y17" s="3" t="inlineStr">
         <is>
-          <t>İki yatak aynı odada; 2 yatak odası yok.</t>
+          <t>Oda, konum ve koşullar doğrulanmalı.</t>
         </is>
       </c>
       <c r="Z17" s="5" t="inlineStr">
@@ -2358,28 +2358,28 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>L23</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Booking</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>2 odalı aydınlık | Val d'Or | La Défense yakınında</t>
+          <t>Le Champs-Elysees - Cité universitaire Paris 14</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>48684</v>
+        <v>58000</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>48685</v>
+        <v>60448</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>1</v>
@@ -2390,67 +2390,61 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Yatak odası 1 kraliçe yatak Oturma odası 1 kanepe</t>
+          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
         </is>
       </c>
       <c r="L18" s="2" t="n">
-        <v>4.91</v>
+        <v>7.7</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>9.4</v>
+        <v>3.3</v>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>Le Val d'Or</t>
+          <t>Gentilly</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>TRAIN L</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T18" s="2" t="n">
-        <v>420</v>
+        <v>460</v>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>yaklaşık</t>
+          <t>kesin</t>
         </is>
       </c>
       <c r="V18" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Saint-Cloud, Fransa</t>
+          <t>18 Rue Dedouvre, 94250 Gentilly, Fransa</t>
         </is>
       </c>
       <c r="W18" s="3" t="inlineStr">
         <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X18" s="2" t="inlineStr">
-        <is>
-          <t>16:00-22:00</t>
-        </is>
-      </c>
+          <t>İade edilmez</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="n"/>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t>1 yatak odası; 2 ayrı oda koşulunu sağlamıyor.</t>
+          <t>250 € depozito; ana fiyat okunamadı; 2 yatak odası yok.</t>
         </is>
       </c>
       <c r="Z18" s="5" t="inlineStr">
@@ -2469,11 +2463,11 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2483,14 +2477,14 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Le Champs-Elysees - Cité universitaire Paris 14</t>
+          <t>Nid Parisien</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>58000</v>
+        <v>56500</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>60448</v>
+        <v>56522</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>1</v>
@@ -2509,24 +2503,24 @@
         </is>
       </c>
       <c r="L19" s="2" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>3.3</v>
+        <v>5.1</v>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>Gentilly</t>
+          <t>Arcueil - Cachan</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -2535,7 +2529,7 @@
         </is>
       </c>
       <c r="T19" s="2" t="n">
-        <v>460</v>
+        <v>290</v>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
@@ -2544,18 +2538,18 @@
       </c>
       <c r="V19" s="3" t="inlineStr">
         <is>
-          <t>18 Rue Dedouvre, 94250 Gentilly, Fransa</t>
+          <t>Rue de la Grange Ory, 94230 Cachan, Fransa</t>
         </is>
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
-          <t>İade edilmez</t>
+          <t>8 Kasım 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X19" s="2" t="n"/>
       <c r="Y19" s="3" t="inlineStr">
         <is>
-          <t>250 € depozito; ana fiyat okunamadı; 2 yatak odası yok.</t>
+          <t>18 yaş; 2 yatak odası yok.</t>
         </is>
       </c>
       <c r="Z19" s="5" t="inlineStr">
@@ -2574,11 +2568,11 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2588,14 +2582,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Nid Parisien</t>
+          <t>T2 Coteau CACHAN</t>
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>56500</v>
+        <v>46000</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>56522</v>
+        <v>46590</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>1</v>
@@ -2610,37 +2604,37 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
+          <t>Yatak Odası 1: 1 çift kişilik yatak ve 1 büyük çift kişilik yatak</t>
         </is>
       </c>
       <c r="L20" s="2" t="n">
-        <v>7.4</v>
+        <v>9</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>Arcueil - Cachan</t>
+          <t>Villejuif - Gustave Roussy</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>METRO 14</t>
         </is>
       </c>
       <c r="T20" s="2" t="n">
-        <v>290</v>
+        <v>820</v>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
@@ -2649,18 +2643,18 @@
       </c>
       <c r="V20" s="3" t="inlineStr">
         <is>
-          <t>Rue de la Grange Ory, 94230 Cachan, Fransa</t>
+          <t>Appartement A 6 Boulevard de la Vanne, 94230 Cachan, Fransa</t>
         </is>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
-          <t>8 Kasım 2026 öncesinde ücretsiz iptal</t>
+          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X20" s="2" t="n"/>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t>18 yaş; 2 yatak odası yok.</t>
+          <t>İki yatak aynı odada; 2 yatak odası yok.</t>
         </is>
       </c>
       <c r="Z20" s="5" t="inlineStr">
@@ -2679,28 +2673,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L23</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Booking</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Cozy studio near RER B</t>
+          <t>2 odalı aydınlık | Val d'Or | La Défense yakınında</t>
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>41200</v>
+        <v>48684</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>41173</v>
+        <v>48685</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>1</v>
@@ -2711,61 +2705,67 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
+          <t>Yatak odası 1 kraliçe yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L21" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>4.91</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="O21" s="2" t="n"/>
+        <v>86</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="P21" s="2" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>16.5</v>
+        <v>9.4</v>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>Palaiseau - Villebon</t>
+          <t>Le Val d'Or</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>TRAIN L</t>
         </is>
       </c>
       <c r="T21" s="2" t="n">
-        <v>550</v>
+        <v>420</v>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>kesin</t>
+          <t>yaklaşık</t>
         </is>
       </c>
       <c r="V21" s="3" t="inlineStr">
         <is>
-          <t>167 Rue de Paris, 91120 Palaiseau, Fransa</t>
+          <t>Tüm kiralık konut, Saint-Cloud, Fransa</t>
         </is>
       </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
-          <t>8 Kasım 2026 öncesinde ücretsiz iptal</t>
-        </is>
-      </c>
-      <c r="X21" s="2" t="n"/>
+          <t>24 saat süreyle ücretsiz iptal.</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>16:00-22:00</t>
+        </is>
+      </c>
       <c r="Y21" s="3" t="inlineStr">
         <is>
-          <t>2 yatak odası yok; daha ucuz başka seçenek var, kişi kapasitesi doğrulanmalı.</t>
+          <t>1 yatak odası; 2 ayrı oda koşulunu sağlamıyor.</t>
         </is>
       </c>
       <c r="Z21" s="5" t="inlineStr">
@@ -2784,11 +2784,11 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2798,14 +2798,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Résidence ROZ 2</t>
+          <t>Parc Montsouris Paris</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>46000</v>
+        <v>62300</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>45614</v>
+        <v>67357</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>1</v>
@@ -2820,37 +2820,37 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 2 çift kişilik yatak</t>
+          <t>Yatak Odası 1: 1 büyük çift kişilik yatak</t>
         </is>
       </c>
       <c r="L22" s="2" t="n">
-        <v>7.9</v>
+        <v>6.4</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>12.7</v>
+        <v>2.6</v>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t>Les Baconnets</t>
+          <t>Montsouris</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>TRAM 3a</t>
         </is>
       </c>
       <c r="T22" s="2" t="n">
-        <v>460</v>
+        <v>190</v>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
@@ -2859,18 +2859,18 @@
       </c>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t>146 Avenue du President Kennedy residence 2, 92160 Antony, Fransa</t>
+          <t>18 Rue Nansouty, 14. Montparnasse, 75014 Paris, Fransa</t>
         </is>
       </c>
       <c r="W22" s="3" t="inlineStr">
         <is>
-          <t>6 Kasım 2026 öncesinde ücretsiz iptal</t>
+          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X22" s="2" t="n"/>
       <c r="Y22" s="3" t="inlineStr">
         <is>
-          <t>İki yatak aynı odada; 2 yatak odası yok.</t>
+          <t>500 € kart depozitosu; ilk fiyat iptal şartı kontrol edilmeli; 2 yatak odası yok.</t>
         </is>
       </c>
       <c r="Z22" s="5" t="inlineStr">
@@ -2889,11 +2889,11 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>L11</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2903,14 +2903,14 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Aparthotel Adagio Access Palaiseau</t>
+          <t>Cozy studio near RER B</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>46200</v>
+        <v>41200</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>46550</v>
+        <v>41173</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>1</v>
@@ -2923,26 +2923,30 @@
       <c r="J23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="3" t="n"/>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
+        </is>
+      </c>
       <c r="L23" s="2" t="n">
-        <v>7.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>244</v>
+        <v>23</v>
       </c>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>15.4</v>
+        <v>16.5</v>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>Palaiseau</t>
+          <t>Palaiseau - Villebon</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -2951,7 +2955,7 @@
         </is>
       </c>
       <c r="T23" s="2" t="n">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
@@ -2960,18 +2964,18 @@
       </c>
       <c r="V23" s="3" t="inlineStr">
         <is>
-          <t>21 Avenue des Allies, 91120 Palaiseau, Fransa</t>
+          <t>167 Rue de Paris, 91120 Palaiseau, Fransa</t>
         </is>
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
-          <t>İade edilmez</t>
+          <t>8 Kasım 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X23" s="2" t="n"/>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>150 € depozito; 18 yaş. Önerilen birim tek yatak odalı daire.</t>
+          <t>2 yatak odası yok; daha ucuz başka seçenek var, kişi kapasitesi doğrulanmalı.</t>
         </is>
       </c>
       <c r="Z23" s="5" t="inlineStr">
@@ -2990,11 +2994,11 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -3004,14 +3008,14 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Parc Montsouris Paris</t>
+          <t>Résidence ROZ 2</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>62300</v>
+        <v>46000</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>67357</v>
+        <v>45614</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>1</v>
@@ -3026,37 +3030,37 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Yatak Odası 1: 1 büyük çift kişilik yatak</t>
+          <t>Yatak Odası 1: 2 çift kişilik yatak</t>
         </is>
       </c>
       <c r="L24" s="2" t="n">
-        <v>6.4</v>
+        <v>7.9</v>
       </c>
       <c r="M24" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>2.6</v>
+        <v>12.7</v>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>Montsouris</t>
+          <t>Les Baconnets</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>TRAM 3a</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T24" s="2" t="n">
-        <v>190</v>
+        <v>460</v>
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
@@ -3065,18 +3069,18 @@
       </c>
       <c r="V24" s="3" t="inlineStr">
         <is>
-          <t>18 Rue Nansouty, 14. Montparnasse, 75014 Paris, Fransa</t>
+          <t>146 Avenue du President Kennedy residence 2, 92160 Antony, Fransa</t>
         </is>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
-          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
+          <t>6 Kasım 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X24" s="2" t="n"/>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>500 € kart depozitosu; ilk fiyat iptal şartı kontrol edilmeli; 2 yatak odası yok.</t>
+          <t>İki yatak aynı odada; 2 yatak odası yok.</t>
         </is>
       </c>
       <c r="Z24" s="5" t="inlineStr">
@@ -3095,11 +3099,11 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L11</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -3109,14 +3113,14 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Le Jardin Edgar Malakoff</t>
+          <t>Aparthotel Adagio Access Palaiseau</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>46800</v>
+        <v>46200</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>46912</v>
+        <v>46550</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>1</v>
@@ -3129,39 +3133,35 @@
       <c r="J25" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
-        </is>
-      </c>
+      <c r="K25" s="3" t="n"/>
       <c r="L25" s="2" t="n">
-        <v>6.2</v>
+        <v>7.3</v>
       </c>
       <c r="M25" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>14</v>
+        <v>244</v>
       </c>
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>3.7</v>
+        <v>15.4</v>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>Malakoff - Plateau De Vanves</t>
+          <t>Palaiseau</t>
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>METRO 13</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T25" s="2" t="n">
-        <v>290</v>
+        <v>520</v>
       </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
@@ -3170,18 +3170,18 @@
       </c>
       <c r="V25" s="3" t="inlineStr">
         <is>
-          <t>3 Rue Edgar Quinet, 92240 Malakoff, Fransa</t>
+          <t>21 Avenue des Allies, 91120 Palaiseau, Fransa</t>
         </is>
       </c>
       <c r="W25" s="3" t="inlineStr">
         <is>
-          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
+          <t>İade edilmez</t>
         </is>
       </c>
       <c r="X25" s="2" t="n"/>
       <c r="Y25" s="3" t="inlineStr">
         <is>
-          <t>250 € kart depozitosu; 18 yaş; 2 yatak odası şartını sağlamıyor.</t>
+          <t>150 € depozito; 18 yaş. Önerilen birim tek yatak odalı daire.</t>
         </is>
       </c>
       <c r="Z25" s="5" t="inlineStr">
@@ -3200,11 +3200,11 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -3214,14 +3214,14 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Séjours &amp; Affaires Massy Atlantis</t>
+          <t>Le Jardin Edgar Malakoff</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>57500</v>
+        <v>46800</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>57602</v>
+        <v>46912</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>1</v>
@@ -3234,35 +3234,39 @@
       <c r="J26" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K26" s="3" t="n"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Yatak Odası 1: 1 çift kişilik yatak</t>
+        </is>
+      </c>
       <c r="L26" s="2" t="n">
-        <v>7.4</v>
+        <v>6.2</v>
       </c>
       <c r="M26" s="2" t="n">
         <v>10</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1472</v>
+        <v>14</v>
       </c>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>14.3</v>
+        <v>3.7</v>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>Massy - Palaiseau</t>
+          <t>Malakoff - Plateau De Vanves</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>METRO 18, RER C, TRAIN V, RER B</t>
+          <t>METRO 13</t>
         </is>
       </c>
       <c r="T26" s="2" t="n">
-        <v>440</v>
+        <v>290</v>
       </c>
       <c r="U26" s="2" t="inlineStr">
         <is>
@@ -3271,34 +3275,135 @@
       </c>
       <c r="V26" s="3" t="inlineStr">
         <is>
-          <t>6 rue Christophe Colomb, 91300 Massy, Fransa</t>
+          <t>3 Rue Edgar Quinet, 92240 Malakoff, Fransa</t>
         </is>
       </c>
       <c r="W26" s="3" t="inlineStr">
         <is>
-          <t>İade edilmez</t>
+          <t>30 Ekim 2026 öncesinde ücretsiz iptal</t>
         </is>
       </c>
       <c r="X26" s="2" t="n"/>
       <c r="Y26" s="3" t="inlineStr">
         <is>
+          <t>250 € kart depozitosu; 18 yaş; 2 yatak odası şartını sağlamıyor.</t>
+        </is>
+      </c>
+      <c r="Z26" s="5" t="inlineStr">
+        <is>
+          <t>aç ↗</t>
+        </is>
+      </c>
+      <c r="AA26" s="5" t="inlineStr">
+        <is>
+          <t>aç ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>L08</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Séjours &amp; Affaires Massy Atlantis</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>57500</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>57602</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>yok</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="2" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>1472</v>
+      </c>
+      <c r="O27" s="2" t="n"/>
+      <c r="P27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="R27" s="3" t="inlineStr">
+        <is>
+          <t>Massy - Palaiseau</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>METRO 18, RER C, TRAIN V, RER B</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>kesin</t>
+        </is>
+      </c>
+      <c r="V27" s="3" t="inlineStr">
+        <is>
+          <t>6 rue Christophe Colomb, 91300 Massy, Fransa</t>
+        </is>
+      </c>
+      <c r="W27" s="3" t="inlineStr">
+        <is>
+          <t>İade edilmez</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="n"/>
+      <c r="Y27" s="3" t="inlineStr">
+        <is>
           <t>150 € kart depozitosu; 18 yaş. Önerilen birim tek yatak odalı daire.</t>
         </is>
       </c>
-      <c r="Z26" s="5" t="inlineStr">
-        <is>
-          <t>aç ↗</t>
-        </is>
-      </c>
-      <c r="AA26" s="5" t="inlineStr">
+      <c r="Z27" s="5" t="inlineStr">
+        <is>
+          <t>aç ↗</t>
+        </is>
+      </c>
+      <c r="AA27" s="5" t="inlineStr">
         <is>
           <t>aç ↗</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA26"/>
-  <conditionalFormatting sqref="B2:B26">
+  <autoFilter ref="A1:AA27"/>
+  <conditionalFormatting sqref="B2:B27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="20"/>
@@ -3361,6 +3466,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3412,17 +3519,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L18</t>
+          <t>L17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
+          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -3430,32 +3537,32 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gurpreet himself gets 5 stars! He was always available and communicative! The apartment... Well, the day before arrival, Gurpreet wrote to me that there was water damage and a wall looks like it. However, the damage was not from 'yesterday', he could have mentioned this, especially since the apartment smelled and was moldy accordingly. Likewise, the walls are like paper. Above the apartment, you could hear trampling </t>
+          <t>In my case, the place was very convenient because of its proximity to the exam center. :)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L18</t>
+          <t>L17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
+          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Decided on this let due to the strength of the reviews. I was contacted 3 days before the holiday to say there was a leak and water damage had occurred and the flat is ok to stay in. Given how casual this was mentioned and also with little time left to find an alternative I agreed to stay. The damp was very bad and appeared to be a long standing problem not something that happened 3 days before. The smell of damp was</t>
+          <t>There was no stay because after seeing the condition of the apartment, we requested a change.</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3579,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -3480,7 +3587,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>In my case, the place was very convenient because of its proximity to the exam center. :)</t>
+          <t>The proximity to the subway is an advantage, but when we first entered the house, there was a strong smell of dampness. This bothered us quite a bit. It improved when we ventilated. Our host couldn't resolve this issue. The good thing was that he was available at all times.</t>
         </is>
       </c>
     </row>
@@ -3497,15 +3604,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>There was no stay because after seeing the condition of the apartment, we requested a change.</t>
+          <t>very well located. BUT - bedroom 3 is actually the living room (so there are 2 bedrooms and not 3) - one bedroom is WITHOUT A WINDOW... how can you ventilate? is it legal? - the basement given as usable is without any windows (!!!), unheated except by a device that stops after 20 minutes and that cannot be restarted - the kitchen is not heated (!)</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3629,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2025-03-20</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -3530,99 +3637,99 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>The proximity to the subway is an advantage, but when we first entered the house, there was a strong smell of dampness. This bothered us quite a bit. It improved when we ventilated. Our host couldn't resolve this issue. The good thing was that he was available at all times.</t>
+          <t>The place has enough rooms for a family to stay, however it’s a bit cluttered and very compact. The alley in between the rooms is very narrow and there is not much space within the rooms as well. The garden however is beautiful. The basement is a nice place to hangout but one has to descend through a very narrow ladder to reach to basement. The cooling system does not let you to heat above 18 degrees, so it was prett</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L17</t>
+          <t>L18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
+          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-11-10</t>
+          <t>2025-08-11</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>very well located. BUT - bedroom 3 is actually the living room (so there are 2 bedrooms and not 3) - one bedroom is WITHOUT A WINDOW... how can you ventilate? is it legal? - the basement given as usable is without any windows (!!!), unheated except by a device that stops after 20 minutes and that cannot be restarted - the kitchen is not heated (!)</t>
+          <t xml:space="preserve">Gurpreet himself gets 5 stars! He was always available and communicative! The apartment... Well, the day before arrival, Gurpreet wrote to me that there was water damage and a wall looks like it. However, the damage was not from 'yesterday', he could have mentioned this, especially since the apartment smelled and was moldy accordingly. Likewise, the walls are like paper. Above the apartment, you could hear trampling </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L17</t>
+          <t>L18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
+          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>The place has enough rooms for a family to stay, however it’s a bit cluttered and very compact. The alley in between the rooms is very narrow and there is not much space within the rooms as well. The garden however is beautiful. The basement is a nice place to hangout but one has to descend through a very narrow ladder to reach to basement. The cooling system does not let you to heat above 18 degrees, so it was prett</t>
+          <t>Decided on this let due to the strength of the reviews. I was contacted 3 days before the holiday to say there was a leak and water damage had occurred and the flat is ok to stay in. Given how casual this was mentioned and also with little time left to find an alternative I agreed to stay. The damp was very bad and appeared to be a long standing problem not something that happened 3 days before. The smell of damp was</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L27</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Teraslı büyüleyici daire - 2 yatak odası/4 kişi - Paris yakınında</t>
+          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">We booked two nights for four people and left the listing the next morning, after only one night. A break-in occurred around 1 a.m. during our stay, which caused us to have a sleepless night and did not allow us to feel safe on the premises. The indoor temperature recorded was 30°C. The host brought us two fans about an hour after our arrival, which I appreciate, but it was not enough to make the nights comfortable. </t>
+          <t>The entrance to the building is at the back, short distance walk to two stations and shops. Close to Notre Dame. The apartment is ok, the drain in the bathroom sink has a very very slow drain. The sheets in one room didn't feel clean. Otherwise the apartment is OK.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>L14</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aile için T3, ulaşım, mağazalar</t>
+          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2025-07-19</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3630,49 +3737,49 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>The apartment is spacious, located on the 4th floor, with an elevator. The kitchen is minimally equipped, with only the most basic amenities. The handle on the bathroom door was broken, not all the lights worked, and one gas burner didn't work. Limited sound insulation, so street noise is clearly audible inside, especially at the front; it is quiet at the back. The center of Paris is easy to reach, by RER or metro, w</t>
+          <t>It was good, easy access to the RER and a safe area</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>L12</t>
+          <t>L27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
+          <t>Teraslı büyüleyici daire - 2 yatak odası/4 kişi - Paris yakınında</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>The entrance to the building is at the back, short distance walk to two stations and shops. Close to Notre Dame. The apartment is ok, the drain in the bathroom sink has a very very slow drain. The sheets in one room didn't feel clean. Otherwise the apartment is OK.</t>
+          <t xml:space="preserve">We booked two nights for four people and left the listing the next morning, after only one night. A break-in occurred around 1 a.m. during our stay, which caused us to have a sleepless night and did not allow us to feel safe on the premises. The indoor temperature recorded was 30°C. The host brought us two fans about an hour after our arrival, which I appreciate, but it was not enough to make the nights comfortable. </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>L12</t>
+          <t>L13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
+          <t>Appartement T3 Antony/Orly 10 dk.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-07-19</t>
+          <t>2025-10-30</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3680,24 +3787,24 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>It was good, easy access to the RER and a safe area</t>
+          <t>Accommodation, quite large and functional. The bedding needs to be reviewed, the cleaning of the dishes too.  HLM neighborhood, quiet Accommodation, clean and linen too</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>L13</t>
+          <t>L15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Appartement T3 Antony/Orly 10 dk.</t>
+          <t>Daire F3 - Arcueil</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -3705,7 +3812,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Accommodation, quite large and functional. The bedding needs to be reviewed, the cleaning of the dishes too.  HLM neighborhood, quiet Accommodation, clean and linen too</t>
+          <t>The apartment itself is nice, and the host is responsive when contacted. However, during my stay there was a very concerning incident: at around 1:00 a.m., someone attempted to enter the apartment using the access code. We had to call the police, and additional security measures were added afterward. Unfortunately, there was also significant noise from the upstairs neighbor, which made it difficult for me to sleep pr</t>
         </is>
       </c>
     </row>
@@ -3722,15 +3829,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>The apartment itself is nice, and the host is responsive when contacted. However, during my stay there was a very concerning incident: at around 1:00 a.m., someone attempted to enter the apartment using the access code. We had to call the police, and additional security measures were added afterward. Unfortunately, there was also significant noise from the upstairs neighbor, which made it difficult for me to sleep pr</t>
+          <t>Unfortunately, a disappointing stay. The accommodation had a lot of ants and, most importantly, a person entered the apartment while we were inside, without waiting for our response. Even though it was due to a mix-up, we felt very uncomfortable and were unable to enjoy the stay with peace of mind. Too bad.</t>
         </is>
       </c>
     </row>
@@ -3747,15 +3854,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Unfortunately, a disappointing stay. The accommodation had a lot of ants and, most importantly, a person entered the apartment while we were inside, without waiting for our response. Even though it was due to a mix-up, we felt very uncomfortable and were unable to enjoy the stay with peace of mind. Too bad.</t>
+          <t>Personally, I won't go back.</t>
         </is>
       </c>
     </row>
@@ -3772,15 +3879,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Personally, I won't go back.</t>
+          <t>The hose was not clean and had rat poop and a mouse running around. Unfortunately, we had to leave an hour after we checked in because of this.</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3904,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -3805,7 +3912,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>The hose was not clean and had rat poop and a mouse running around. Unfortunately, we had to leave an hour after we checked in because of this.</t>
+          <t>We arrived at this accommodation which had not been cleaned, still the sheets of the old tenant, as well as pubic hair and bathroom hair, disgusting, no towels to dry yourself, the trash had not been emptied. In short, no one had taken care of this apartment and the host never answered me. I had to contact Airbnb support to find a solution. And while waiting for this solution, I had to wait outside in the rain at 9 p</t>
         </is>
       </c>
     </row>
@@ -3822,15 +3929,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>We arrived at this accommodation which had not been cleaned, still the sheets of the old tenant, as well as pubic hair and bathroom hair, disgusting, no towels to dry yourself, the trash had not been emptied. In short, no one had taken care of this apartment and the host never answered me. I had to contact Airbnb support to find a solution. And while waiting for this solution, I had to wait outside in the rain at 9 p</t>
+          <t xml:space="preserve">I booked this apartment a couple of months prior. I had asked the host as soon as I booked if we could do a late check out and I got a response a couple of weeks before the day of the booking. I didn’t mind since the response was before and he was flexible and let us check out later which we’re grateful for. I usually don’t leave bad reviews but what upset me is that the instructions were unclear on checking in. All </t>
         </is>
       </c>
     </row>
@@ -3847,15 +3954,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2025-08-06</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">I booked this apartment a couple of months prior. I had asked the host as soon as I booked if we could do a late check out and I got a response a couple of weeks before the day of the booking. I didn’t mind since the response was before and he was flexible and let us check out later which we’re grateful for. I usually don’t leave bad reviews but what upset me is that the instructions were unclear on checking in. All </t>
+          <t>Good accommodation suitable for a short trip to Paris  Well served by the RER B Downside, you can hear the neighbors upstairs a lot when the place is occupied</t>
         </is>
       </c>
     </row>
@@ -3872,15 +3979,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025-08-06</t>
+          <t>2025-07-07</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Good accommodation suitable for a short trip to Paris  Well served by the RER B Downside, you can hear the neighbors upstairs a lot when the place is occupied</t>
+          <t>I am disappointed with the long full trash, bathroom towels on the floor, I turned on the hot water tank to shower because the water when I arrived was cold. Bed not made. Honestly, I would have been better off going to the hotel.</t>
         </is>
       </c>
     </row>
@@ -3897,15 +4004,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2025-07-07</t>
+          <t>2025-04-22</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>I am disappointed with the long full trash, bathroom towels on the floor, I turned on the hot water tank to shower because the water when I arrived was cold. Bed not made. Honestly, I would have been better off going to the hotel.</t>
+          <t xml:space="preserve">the place looks like the pictures. However, during our stay there was a party upstairs. The screams and jumping from the party were so loud that we it felt like the ceiling ws going to fall on us. when we contacted the host he responded thr messages but he wasn't nearby; we were stranded without been able to sleep with a baby until pass 4 am. upstairs is his Airbnb as well. There was a large group of people upstairs </t>
         </is>
       </c>
     </row>
@@ -3922,32 +4029,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2025-04-22</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">the place looks like the pictures. However, during our stay there was a party upstairs. The screams and jumping from the party were so loud that we it felt like the ceiling ws going to fall on us. when we contacted the host he responded thr messages but he wasn't nearby; we were stranded without been able to sleep with a baby until pass 4 am. upstairs is his Airbnb as well. There was a large group of people upstairs </t>
+          <t>Very responsive and warm host, very attentive.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>L15</t>
+          <t>L14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Daire F3 - Arcueil</t>
+          <t>Aile için T3, ulaşım, mağazalar</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -3955,7 +4062,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Very responsive and warm host, very attentive.</t>
+          <t>The apartment is spacious, located on the 4th floor, with an elevator. The kitchen is minimally equipped, with only the most basic amenities. The handle on the bathroom door was broken, not all the lights worked, and one gas burner didn't work. Limited sound insulation, so street noise is clearly audible inside, especially at the front; it is quiet at the back. The center of Paris is easy to reach, by RER or metro, w</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4136,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oluşturulma: 2026-10-27 · 13–22 Kasım 2026. 9 gece. 3 yetişkin · bütçe 65.000 TL</t>
+          <t>Oluşturulma: 2026-10-28 · 13–22 Kasım 2026. 9 gece. 3 yetişkin · bütçe 65.000 TL</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4150,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Skor (0–100), önem sırasıyla: 2 ayrı yatak odası 40 (salondaki çekyat sayılmaz; oda dökümü yoksa 32, şüpheliyse 18), puan 15 + yorumlar 10 (her 3★ altı yorum −2,5, izinsiz giriş iddiası −5), Mines'e süre 20 (15 dk tam, 55 dk sıfır, 1 saat üstü −5), fiyat 15. Fiyatı olmayan ilan en çok 45.</t>
+          <t>Skor (0–100), önem sırasıyla: 2 ayrı yatak odası 40 (salondaki çekyat sayılmaz; oda dökümü yoksa 32, şüpheliyse 18); puan 15 (az yorumlu ilanın puanı platform ortalamasına çekilir) + yorumlar 10 (son 2 yılın 3★ altı yorumları toplam yorumun %8'ine ulaşınca 0; izinsiz giriş iddiası −5); Mines'e kapıdan kapıya süre 20 (15 dk tam, 40 dk sıfır, sonrası dakika başı −0,5); fiyat: 65.000 TL bütçe içinde 3–15, bütçe üstü her 1.000 TL −2 (en çok −15). Süreler elle girildi (data/transit_manual.csv).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
L28 transit time 26 min
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/Paris_konaklama_v2.xlsx
+++ b/out/Paris_konaklama_v2.xlsx
@@ -1068,11 +1068,11 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>L17</t>
+          <t>L28</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1082,14 +1082,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
+          <t>L'Écrin Parisien • T3 Design • Le Bourget • CDG Havalimanı</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>71934</v>
+        <v>72174</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>61880</v>
+        <v>62442</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>2</v>
@@ -1100,43 +1100,43 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 çift kişilik yatak</t>
+          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak Oturma odası 1 kanepe</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>4.63</v>
+        <v>4.94</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>4</v>
+        <v>11.6</v>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>Laplace</t>
+          <t>Le Bourget</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>RER B, TRAM 11</t>
         </is>
       </c>
       <c r="T6" s="2" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
@@ -1145,22 +1145,18 @@
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t>Tüm villa, Arcueil, Fransa</t>
+          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
         </is>
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 30 Ekim</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="inlineStr">
-        <is>
-          <t>15:00-23:00</t>
-        </is>
-      </c>
+          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="n"/>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>Önceki tabloda A07; Laplace RER 2–3 dk; Ağustos 2026’da evin durumu hakkında olumsuz değerlendirme var.</t>
+          <t>Kullanıcı sonradan ekledi (28.10.2026).</t>
         </is>
       </c>
       <c r="Z6" s="5" t="inlineStr">
@@ -1183,7 +1179,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>L18</t>
+          <t>L17</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1193,14 +1189,14 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
+          <t>Bahçe evi, otopark, 3 dakika RER, 1 km Paris</t>
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>70047</v>
+        <v>71934</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>60723</v>
+        <v>61880</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>2</v>
@@ -1215,39 +1211,39 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 çift kişilik yatak</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>4.88</v>
+        <v>4.63</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>11.4</v>
+        <v>4</v>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>Le Bourget</t>
+          <t>Laplace</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>RER B, TRAM 11</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T7" s="2" t="n">
-        <v>260</v>
+        <v>130</v>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
@@ -1256,22 +1252,22 @@
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
+          <t>Tüm villa, Arcueil, Fransa</t>
         </is>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+          <t>Ücretsiz iptal son gün: 30 Ekim</t>
         </is>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>14:00-22:00</t>
+          <t>15:00-23:00</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>Önceki tabloda A02; misafir yorumuna göre RER 3 dk; 12 Kasım ücretsiz iptal.</t>
+          <t>Önceki tabloda A07; Laplace RER 2–3 dk; Ağustos 2026’da evin durumu hakkında olumsuz değerlendirme var.</t>
         </is>
       </c>
       <c r="Z7" s="5" t="inlineStr">
@@ -1290,11 +1286,11 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>L12</t>
+          <t>L18</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1304,57 +1300,61 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
+          <t>Yeni Lux 60m² Tüm apart+Klima Paris yakınında</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>66832</v>
+        <v>70047</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>58136</v>
+        <v>60723</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>doğrulanmalı</t>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>onaylı</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="3" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="n">
-        <v>4.9</v>
+        <v>4.88</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>129</v>
+        <v>90</v>
       </c>
       <c r="O8" s="2" t="n">
         <v>2</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>La Croix de Berny</t>
+          <t>Le Bourget</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>RER B, TRAM 10</t>
+          <t>RER B, TRAM 11</t>
         </is>
       </c>
       <c r="T8" s="2" t="n">
-        <v>290</v>
+        <v>260</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
@@ -1363,14 +1363,22 @@
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>Tüm site içi konut, Antony, Fransa</t>
-        </is>
-      </c>
-      <c r="W8" s="3" t="n"/>
-      <c r="X8" s="2" t="n"/>
+          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="inlineStr">
+        <is>
+          <t>Ücretsiz iptal son gün: 12 Kasım</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>14:00-22:00</t>
+        </is>
+      </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>Arama fiyatı 9 gece için tüm ücretler dâhil gösteriliyor; oda ve koşullar incelenmeli.</t>
+          <t>Önceki tabloda A02; misafir yorumuna göre RER 3 dk; 12 Kasım ücretsiz iptal.</t>
         </is>
       </c>
       <c r="Z8" s="5" t="inlineStr">
@@ -1393,7 +1401,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>L27</t>
+          <t>L12</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1403,61 +1411,57 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Teraslı büyüleyici daire - 2 yatak odası/4 kişi - Paris yakınında</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>52341</v>
+          <t>Paris + Orly Havalimanı'na yakın daire + otopark</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>66832</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>48436</v>
+        <v>58136</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>onaylı</t>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>doğrulanmalı</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K9" s="3" t="n"/>
       <c r="L9" s="2" t="n">
-        <v>4.53</v>
+        <v>4.9</v>
       </c>
       <c r="M9" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>Mairie d'Aubervilliers</t>
+          <t>La Croix de Berny</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>METRO 12</t>
+          <t>RER B, TRAM 10</t>
         </is>
       </c>
       <c r="T9" s="2" t="n">
-        <v>400</v>
+        <v>290</v>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
@@ -1466,22 +1470,14 @@
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Aubervilliers, Fransa</t>
-        </is>
-      </c>
-      <c r="W9" s="3" t="inlineStr">
-        <is>
-          <t>24 saat süreyle ücretsiz iptal.</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>16:00-23:00</t>
-        </is>
-      </c>
+          <t>Tüm site içi konut, Antony, Fransa</t>
+        </is>
+      </c>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="2" t="n"/>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>30 m²; her odada çift kişilik yatak. Bir yorumda gece izinsiz giriş iddiası var; ücretsiz iptal ilk 24 saatle sınırlı.</t>
+          <t>Arama fiyatı 9 gece için tüm ücretler dâhil gösteriliyor; oda ve koşullar incelenmeli.</t>
         </is>
       </c>
       <c r="Z9" s="5" t="inlineStr">
@@ -1500,11 +1496,11 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>L13</t>
+          <t>L27</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1514,57 +1510,61 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Appartement T3 Antony/Orly 10 dk.</t>
+          <t>Teraslı büyüleyici daire - 2 yatak odası/4 kişi - Paris yakınında</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>62401</v>
+        <v>52341</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>54348</v>
+        <v>48436</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>doğrulanmalı</t>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>onaylı</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K10" s="3" t="n"/>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="n">
-        <v>4.57</v>
+        <v>4.53</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>Parc de Sceaux</t>
+          <t>Mairie d'Aubervilliers</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>RER B</t>
+          <t>METRO 12</t>
         </is>
       </c>
       <c r="T10" s="2" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="V10" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Antony, Fransa</t>
+          <t>Tüm kiralık konut, Aubervilliers, Fransa</t>
         </is>
       </c>
       <c r="W10" s="3" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>17:00-23:00</t>
+          <t>16:00-23:00</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t>RER B Parc de Sceaux: ilanda 5 dakika deniyor, yürüyüş olup olmadığı teyit edilmeli.</t>
+          <t>30 m²; her odada çift kişilik yatak. Bir yorumda gece izinsiz giriş iddiası var; ücretsiz iptal ilk 24 saatle sınırlı.</t>
         </is>
       </c>
       <c r="Z10" s="5" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>L16</t>
+          <t>L13</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1621,61 +1621,57 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Montmartre'ın göbeğinde ferah ve aydınlık daire</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>66801</v>
+          <t>Appartement T3 Antony/Orly 10 dk.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>62401</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>57852</v>
+        <v>54348</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>onaylı</t>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>doğrulanmalı</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
-        </is>
-      </c>
+      <c r="K11" s="3" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>4.44</v>
+        <v>4.57</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>4.3</v>
+        <v>8.5</v>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>Abbesses</t>
+          <t>Parc de Sceaux</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>METRO 12</t>
+          <t>RER B</t>
         </is>
       </c>
       <c r="T11" s="2" t="n">
-        <v>210</v>
+        <v>360</v>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
@@ -1684,7 +1680,7 @@
       </c>
       <c r="V11" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Paris, Fransa</t>
+          <t>Tüm kiralık konut, Antony, Fransa</t>
         </is>
       </c>
       <c r="W11" s="3" t="inlineStr">
@@ -1694,12 +1690,12 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>15:00-21:00</t>
+          <t>17:00-23:00</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>Oda düzeni, yorumlar ve ulaşım doğrulanmalı.</t>
+          <t>RER B Parc de Sceaux: ilanda 5 dakika deniyor, yürüyüş olup olmadığı teyit edilmeli.</t>
         </is>
       </c>
       <c r="Z11" s="5" t="inlineStr">
@@ -1718,11 +1714,11 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>L28</t>
+          <t>L16</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1732,14 +1728,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>L'Écrin Parisien • T3 Design • Le Bourget • CDG Havalimanı</t>
+          <t>Montmartre'ın göbeğinde ferah ve aydınlık daire</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>72174</v>
+        <v>66801</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>62442</v>
+        <v>57852</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>2</v>
@@ -1750,41 +1746,43 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>1. yatak odası 1 çift kişilik yatak 2. yatak odası 1 çift kişilik yatak Oturma odası 1 kanepe</t>
+          <t>1. yatak odası 1 kraliçe yatak 2. yatak odası 1 kraliçe yatak</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>4.94</v>
+        <v>4.44</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>5</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P12" s="2" t="n"/>
+      <c r="P12" s="2" t="n">
+        <v>36</v>
+      </c>
       <c r="Q12" s="2" t="n">
-        <v>11.6</v>
+        <v>4.3</v>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>Le Bourget</t>
+          <t>Abbesses</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>RER B, TRAM 11</t>
+          <t>METRO 12</t>
         </is>
       </c>
       <c r="T12" s="2" t="n">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
@@ -1793,18 +1791,22 @@
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t>Tüm kiralık konut, Le Bourget, Fransa</t>
+          <t>Tüm kiralık konut, Paris, Fransa</t>
         </is>
       </c>
       <c r="W12" s="3" t="inlineStr">
         <is>
-          <t>Ücretsiz iptal son gün: 12 Kasım</t>
-        </is>
-      </c>
-      <c r="X12" s="2" t="n"/>
+          <t>24 saat süreyle ücretsiz iptal.</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>15:00-21:00</t>
+        </is>
+      </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>Kullanıcı sonradan ekledi (28.10.2026).</t>
+          <t>Oda düzeni, yorumlar ve ulaşım doğrulanmalı.</t>
         </is>
       </c>
       <c r="Z12" s="5" t="inlineStr">

</xml_diff>